<commit_message>
Full equip suitability and ex slots
Signed-off-by: ibicdlcod <504161487@qq.com>
</commit_message>
<xml_diff>
--- a/doc/ship/Ship.xlsx
+++ b/doc/ship/Ship.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GuoMuoRuoProject\doc\ship\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8216670-8736-4F36-ACAF-C1FBC38E2E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5DABA7-B04F-4802-9BF6-8F19A56033EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Ship" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ship!$A$2:$BJ$944</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ship!$A$2:$BL$944</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21416" uniqueCount="2844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21510" uniqueCount="2858">
   <si>
     <t>id</t>
   </si>
@@ -8641,6 +8641,62 @@
   </si>
   <si>
     <t>6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>secgunex</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>22</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>54</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>customflags</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>radarex</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>20000000</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>10</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>toku4</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -8939,7 +8995,7 @@
     <col min="16384" max="16384" width="10.46484375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9108,8 +9164,17 @@
       <c r="BJ1" s="3" t="s">
         <v>2786</v>
       </c>
-    </row>
-    <row r="2" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK1" s="3" t="s">
+        <v>2786</v>
+      </c>
+      <c r="BL1" s="3" t="s">
+        <v>2851</v>
+      </c>
+      <c r="BM1" s="3" t="s">
+        <v>2851</v>
+      </c>
+    </row>
+    <row r="2" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -9296,8 +9361,17 @@
       <c r="BJ2" s="3" t="s">
         <v>2840</v>
       </c>
-    </row>
-    <row r="3" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK2" s="3" t="s">
+        <v>2844</v>
+      </c>
+      <c r="BL2" s="3" t="s">
+        <v>2852</v>
+      </c>
+      <c r="BM2" s="3" t="s">
+        <v>2857</v>
+      </c>
+    </row>
+    <row r="3" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <f>HEX2DEC(D3)</f>
         <v>169411328</v>
@@ -9380,8 +9454,11 @@
       <c r="BJ3" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="4" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK3" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <f>HEX2DEC(D4)</f>
         <v>186188544</v>
@@ -9450,7 +9527,7 @@
         <v>2841</v>
       </c>
     </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <f>HEX2DEC(D5)</f>
         <v>202965760</v>
@@ -9525,7 +9602,7 @@
         <v>2843</v>
       </c>
     </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <f>HEX2DEC(D6)</f>
         <v>253105920</v>
@@ -9636,7 +9713,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <f>HEX2DEC(D7)</f>
         <v>253105921</v>
@@ -9750,7 +9827,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <f>HEX2DEC(D8)</f>
         <v>269549825</v>
@@ -9855,7 +9932,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <f>HEX2DEC(D9)</f>
         <v>269549826</v>
@@ -9960,7 +10037,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <f>HEX2DEC(D10)</f>
         <v>269549827</v>
@@ -10065,7 +10142,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <f>HEX2DEC(D11)</f>
         <v>269549828</v>
@@ -10170,7 +10247,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <f>HEX2DEC(D12)</f>
         <v>269550081</v>
@@ -10275,7 +10352,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <f>HEX2DEC(D13)</f>
         <v>269550082</v>
@@ -10380,7 +10457,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <f>HEX2DEC(D14)</f>
         <v>269550083</v>
@@ -10485,7 +10562,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <f>HEX2DEC(D15)</f>
         <v>269550087</v>
@@ -10590,7 +10667,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <f>HEX2DEC(D16)</f>
         <v>269550089</v>
@@ -20359,7 +20436,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="113" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A113" s="2">
         <f>HEX2DEC(D113)</f>
         <v>269617411</v>
@@ -20467,7 +20544,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="114" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A114" s="2">
         <f>HEX2DEC(D114)</f>
         <v>269617412</v>
@@ -20575,7 +20652,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="115" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A115" s="2">
         <f>HEX2DEC(D115)</f>
         <v>269617413</v>
@@ -20683,7 +20760,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="116" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A116" s="2">
         <f>HEX2DEC(D116)</f>
         <v>269617414</v>
@@ -20791,7 +20868,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="117" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A117" s="2">
         <f>HEX2DEC(D117)</f>
         <v>269617417</v>
@@ -20899,7 +20976,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="118" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A118" s="2">
         <f>HEX2DEC(D118)</f>
         <v>269617418</v>
@@ -21007,7 +21084,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="119" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A119" s="2">
         <f>HEX2DEC(D119)</f>
         <v>269617419</v>
@@ -21115,7 +21192,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="120" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A120" s="2">
         <f>HEX2DEC(D120)</f>
         <v>269617420</v>
@@ -21223,7 +21300,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="121" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A121" s="2">
         <f>HEX2DEC(D121)</f>
         <v>269617421</v>
@@ -21331,7 +21408,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="122" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A122" s="2">
         <f>HEX2DEC(D122)</f>
         <v>269617422</v>
@@ -21439,7 +21516,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="123" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A123" s="2">
         <f>HEX2DEC(D123)</f>
         <v>269617423</v>
@@ -21546,8 +21623,9 @@
       <c r="AI123" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="124" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BK123" s="5"/>
+    </row>
+    <row r="124" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A124" s="2">
         <f>HEX2DEC(D124)</f>
         <v>269617424</v>
@@ -21654,8 +21732,9 @@
       <c r="AI124" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="125" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BK124" s="5"/>
+    </row>
+    <row r="125" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A125" s="2">
         <f>HEX2DEC(D125)</f>
         <v>269617425</v>
@@ -21762,8 +21841,9 @@
       <c r="AI125" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="126" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BK125" s="5"/>
+    </row>
+    <row r="126" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A126" s="2">
         <f>HEX2DEC(D126)</f>
         <v>269617426</v>
@@ -21870,8 +21950,9 @@
       <c r="AI126" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="127" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BK126" s="5"/>
+    </row>
+    <row r="127" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A127" s="2">
         <f>HEX2DEC(D127)</f>
         <v>269617427</v>
@@ -21978,8 +22059,9 @@
       <c r="AI127" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="128" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BK127" s="5"/>
+    </row>
+    <row r="128" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A128" s="2">
         <f>HEX2DEC(D128)</f>
         <v>269617665</v>
@@ -22086,8 +22168,9 @@
       <c r="AI128" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="129" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK128" s="5"/>
+    </row>
+    <row r="129" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A129" s="2">
         <f>HEX2DEC(D129)</f>
         <v>269617921</v>
@@ -22194,8 +22277,9 @@
       <c r="AI129" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="130" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK129" s="5"/>
+    </row>
+    <row r="130" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A130" s="2">
         <f>HEX2DEC(D130)</f>
         <v>269617922</v>
@@ -22302,8 +22386,9 @@
       <c r="AI130" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="131" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK130" s="5"/>
+    </row>
+    <row r="131" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A131" s="2">
         <f>HEX2DEC(D131)</f>
         <v>269617923</v>
@@ -22410,8 +22495,9 @@
       <c r="AI131" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="132" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK131" s="5"/>
+    </row>
+    <row r="132" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A132" s="2">
         <f>HEX2DEC(D132)</f>
         <v>269617924</v>
@@ -22518,8 +22604,9 @@
       <c r="AI132" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="133" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK132" s="5"/>
+    </row>
+    <row r="133" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A133" s="2">
         <f>HEX2DEC(D133)</f>
         <v>269617928</v>
@@ -22626,8 +22713,9 @@
       <c r="AI133" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="134" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK133" s="5"/>
+    </row>
+    <row r="134" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A134" s="2">
         <f>HEX2DEC(D134)</f>
         <v>269618177</v>
@@ -22728,8 +22816,9 @@
       <c r="AI134" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="135" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK134" s="5"/>
+    </row>
+    <row r="135" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A135" s="2">
         <f>HEX2DEC(D135)</f>
         <v>269618178</v>
@@ -22830,8 +22919,9 @@
       <c r="AI135" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="136" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK135" s="5"/>
+    </row>
+    <row r="136" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A136" s="2">
         <f>HEX2DEC(D136)</f>
         <v>269618179</v>
@@ -22932,8 +23022,9 @@
       <c r="AI136" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="137" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK136" s="5"/>
+    </row>
+    <row r="137" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A137" s="2">
         <f>HEX2DEC(D137)</f>
         <v>269618180</v>
@@ -23034,8 +23125,9 @@
       <c r="AI137" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="138" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK137" s="5"/>
+    </row>
+    <row r="138" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A138" s="2">
         <f>HEX2DEC(D138)</f>
         <v>269618183</v>
@@ -23136,8 +23228,9 @@
       <c r="AI138" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="139" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK138" s="5"/>
+    </row>
+    <row r="139" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A139" s="2">
         <f>HEX2DEC(D139)</f>
         <v>269618187</v>
@@ -23238,8 +23331,9 @@
       <c r="AI139" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="140" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BK139" s="5"/>
+    </row>
+    <row r="140" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A140" s="2">
         <f>HEX2DEC(D140)</f>
         <v>269680897</v>
@@ -23337,7 +23431,7 @@
       </c>
       <c r="XFD140" s="4"/>
     </row>
-    <row r="141" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A141" s="2">
         <f>HEX2DEC(D141)</f>
         <v>269680898</v>
@@ -23435,7 +23529,7 @@
       </c>
       <c r="XFD141" s="4"/>
     </row>
-    <row r="142" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A142" s="2">
         <f>HEX2DEC(D142)</f>
         <v>269681153</v>
@@ -23535,7 +23629,7 @@
       </c>
       <c r="XFD142" s="4"/>
     </row>
-    <row r="143" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A143" s="2">
         <f>HEX2DEC(D143)</f>
         <v>269681154</v>
@@ -23638,7 +23732,7 @@
       </c>
       <c r="XFD143" s="4"/>
     </row>
-    <row r="144" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A144" s="2">
         <f>HEX2DEC(D144)</f>
         <v>269681155</v>
@@ -23738,7 +23832,7 @@
       </c>
       <c r="XFD144" s="4"/>
     </row>
-    <row r="145" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A145" s="2">
         <f>HEX2DEC(D145)</f>
         <v>269681156</v>
@@ -23838,7 +23932,7 @@
       </c>
       <c r="XFD145" s="4"/>
     </row>
-    <row r="146" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A146" s="2">
         <f>HEX2DEC(D146)</f>
         <v>269681157</v>
@@ -23941,7 +24035,7 @@
       </c>
       <c r="XFD146" s="4"/>
     </row>
-    <row r="147" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A147" s="2">
         <f>HEX2DEC(D147)</f>
         <v>269681409</v>
@@ -24041,7 +24135,7 @@
       </c>
       <c r="XFD147" s="4"/>
     </row>
-    <row r="148" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A148" s="2">
         <f>HEX2DEC(D148)</f>
         <v>269681410</v>
@@ -24141,7 +24235,7 @@
       </c>
       <c r="XFD148" s="4"/>
     </row>
-    <row r="149" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A149" s="2">
         <f>HEX2DEC(D149)</f>
         <v>269681411</v>
@@ -24241,7 +24335,7 @@
       </c>
       <c r="XFD149" s="4"/>
     </row>
-    <row r="150" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A150" s="2">
         <f>HEX2DEC(D150)</f>
         <v>269681412</v>
@@ -24341,7 +24435,7 @@
       </c>
       <c r="XFD150" s="4"/>
     </row>
-    <row r="151" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A151" s="2">
         <f>HEX2DEC(D151)</f>
         <v>269681413</v>
@@ -24441,7 +24535,7 @@
       </c>
       <c r="XFD151" s="4"/>
     </row>
-    <row r="152" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A152" s="2">
         <f>HEX2DEC(D152)</f>
         <v>269681414</v>
@@ -24542,9 +24636,10 @@
       <c r="BJ152" s="6" t="s">
         <v>2842</v>
       </c>
+      <c r="BK152" s="1"/>
       <c r="XFD152" s="4"/>
     </row>
-    <row r="153" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A153" s="2">
         <f>HEX2DEC(D153)</f>
         <v>269681665</v>
@@ -24642,9 +24737,10 @@
       <c r="AI153" s="4">
         <v>250</v>
       </c>
+      <c r="BK153" s="1"/>
       <c r="XFD153" s="4"/>
     </row>
-    <row r="154" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A154" s="2">
         <f>HEX2DEC(D154)</f>
         <v>269681666</v>
@@ -24742,9 +24838,10 @@
       <c r="AI154" s="4">
         <v>250</v>
       </c>
+      <c r="BK154" s="1"/>
       <c r="XFD154" s="4"/>
     </row>
-    <row r="155" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A155" s="2">
         <f>HEX2DEC(D155)</f>
         <v>269681667</v>
@@ -24842,9 +24939,10 @@
       <c r="AI155" s="4">
         <v>250</v>
       </c>
+      <c r="BK155" s="1"/>
       <c r="XFD155" s="4"/>
     </row>
-    <row r="156" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A156" s="2">
         <f>HEX2DEC(D156)</f>
         <v>269681921</v>
@@ -24943,9 +25041,10 @@
       <c r="AI156" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="BK156" s="1"/>
       <c r="XFD156" s="4"/>
     </row>
-    <row r="157" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A157" s="2">
         <f>HEX2DEC(D157)</f>
         <v>269682177</v>
@@ -25052,9 +25151,12 @@
       <c r="AI157" s="5" t="s">
         <v>759</v>
       </c>
+      <c r="BK157" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD157" s="4"/>
     </row>
-    <row r="158" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A158" s="2">
         <f>HEX2DEC(D158)</f>
         <v>269682178</v>
@@ -25161,9 +25263,12 @@
       <c r="AI158" s="5" t="s">
         <v>759</v>
       </c>
+      <c r="BK158" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD158" s="4"/>
     </row>
-    <row r="159" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A159" s="2">
         <f>HEX2DEC(D159)</f>
         <v>269682179</v>
@@ -25270,9 +25375,12 @@
       <c r="AI159" s="5" t="s">
         <v>759</v>
       </c>
+      <c r="BK159" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD159" s="4"/>
     </row>
-    <row r="160" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A160" s="2">
         <f>HEX2DEC(D160)</f>
         <v>269682180</v>
@@ -25379,9 +25487,12 @@
       <c r="AI160" s="5" t="s">
         <v>759</v>
       </c>
+      <c r="BK160" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD160" s="4"/>
     </row>
-    <row r="161" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A161" s="2">
         <f>HEX2DEC(D161)</f>
         <v>269682433</v>
@@ -25485,9 +25596,12 @@
       <c r="AI161" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="BK161" s="3" t="s">
+        <v>2846</v>
+      </c>
       <c r="XFD161" s="4"/>
     </row>
-    <row r="162" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A162" s="2">
         <f>HEX2DEC(D162)</f>
         <v>269684994</v>
@@ -25585,9 +25699,10 @@
       <c r="BE162" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK162" s="3"/>
       <c r="XFD162" s="4"/>
     </row>
-    <row r="163" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A163" s="2">
         <f>HEX2DEC(D163)</f>
         <v>269685249</v>
@@ -25691,9 +25806,10 @@
       <c r="BE163" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK163" s="3"/>
       <c r="XFD163" s="4"/>
     </row>
-    <row r="164" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A164" s="2">
         <f>HEX2DEC(D164)</f>
         <v>269685250</v>
@@ -25797,9 +25913,10 @@
       <c r="BE164" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK164" s="3"/>
       <c r="XFD164" s="4"/>
     </row>
-    <row r="165" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A165" s="2">
         <f>HEX2DEC(D165)</f>
         <v>269701377</v>
@@ -25900,9 +26017,10 @@
       <c r="BE165" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK165" s="1"/>
       <c r="XFD165" s="4"/>
     </row>
-    <row r="166" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A166" s="2">
         <f>HEX2DEC(D166)</f>
         <v>269701633</v>
@@ -26000,9 +26118,10 @@
       <c r="BE166" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK166" s="1"/>
       <c r="XFD166" s="4"/>
     </row>
-    <row r="167" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A167" s="2">
         <f>HEX2DEC(D167)</f>
         <v>269701634</v>
@@ -26100,9 +26219,10 @@
       <c r="BE167" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK167" s="1"/>
       <c r="XFD167" s="4"/>
     </row>
-    <row r="168" spans="1:57 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A168" s="2">
         <f>HEX2DEC(D168)</f>
         <v>269701891</v>
@@ -26203,9 +26323,10 @@
       <c r="BE168" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK168" s="1"/>
       <c r="XFD168" s="4"/>
     </row>
-    <row r="169" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A169" s="2">
         <f>HEX2DEC(D169)</f>
         <v>269746433</v>
@@ -26304,7 +26425,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="170" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A170" s="2">
         <f>HEX2DEC(D170)</f>
         <v>269746434</v>
@@ -26403,7 +26524,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="171" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A171" s="2">
         <f>HEX2DEC(D171)</f>
         <v>269746689</v>
@@ -26502,7 +26623,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="172" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A172" s="2">
         <f>HEX2DEC(D172)</f>
         <v>269746690</v>
@@ -26601,7 +26722,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="173" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A173" s="2">
         <f>HEX2DEC(D173)</f>
         <v>269746945</v>
@@ -26700,7 +26821,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="174" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A174" s="2">
         <f>HEX2DEC(D174)</f>
         <v>269746946</v>
@@ -26799,7 +26920,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="175" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A175" s="2">
         <f>HEX2DEC(D175)</f>
         <v>269746947</v>
@@ -26898,7 +27019,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="176" spans="1:57 16384:16384" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A176" s="2">
         <f>HEX2DEC(D176)</f>
         <v>269746948</v>
@@ -29718,7 +29839,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="209" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A209" s="2">
         <f>HEX2DEC(D209)</f>
         <v>269881857</v>
@@ -29814,7 +29935,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="210" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="210" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A210" s="2">
         <f>HEX2DEC(D210)</f>
         <v>269882113</v>
@@ -29916,7 +30037,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="211" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A211" s="2">
         <f>HEX2DEC(D211)</f>
         <v>269882369</v>
@@ -30018,7 +30139,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="212" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="212" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A212" s="2">
         <f>HEX2DEC(D212)</f>
         <v>269882370</v>
@@ -30120,7 +30241,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="213" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="213" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A213" s="2">
         <f>HEX2DEC(D213)</f>
         <v>269882625</v>
@@ -30222,7 +30343,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="214" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="214" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A214" s="2">
         <f>HEX2DEC(D214)</f>
         <v>269882626</v>
@@ -30324,7 +30445,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="215" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="215" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A215" s="2">
         <f>HEX2DEC(D215)</f>
         <v>269891329</v>
@@ -30435,7 +30556,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="216" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A216" s="2">
         <f>HEX2DEC(D216)</f>
         <v>269891330</v>
@@ -30546,7 +30667,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="217" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="217" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A217" s="2">
         <f>HEX2DEC(D217)</f>
         <v>269891332</v>
@@ -30663,7 +30784,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="218" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="218" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A218" s="2">
         <f>HEX2DEC(D218)</f>
         <v>269894913</v>
@@ -30707,8 +30828,11 @@
       <c r="N218" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="219" spans="1:51" x14ac:dyDescent="0.4">
+      <c r="BK218" s="3" t="s">
+        <v>2846</v>
+      </c>
+    </row>
+    <row r="219" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A219" s="2">
         <f>HEX2DEC(D219)</f>
         <v>269943041</v>
@@ -30753,7 +30877,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="220" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="220" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A220" s="2">
         <f>HEX2DEC(D220)</f>
         <v>269943298</v>
@@ -30798,7 +30922,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="221" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="221" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A221" s="2">
         <f>HEX2DEC(D221)</f>
         <v>269943811</v>
@@ -30843,7 +30967,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="222" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="222" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A222" s="2">
         <f>HEX2DEC(D222)</f>
         <v>269943815</v>
@@ -30888,7 +31012,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="223" spans="1:51" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A223" s="2">
         <f>HEX2DEC(D223)</f>
         <v>269943825</v>
@@ -30932,8 +31056,11 @@
       <c r="N223" s="3" t="s">
         <v>568</v>
       </c>
-    </row>
-    <row r="224" spans="1:51" x14ac:dyDescent="0.4">
+      <c r="BM223" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="224" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A224" s="2">
         <f>HEX2DEC(D224)</f>
         <v>269943874</v>
@@ -30977,8 +31104,11 @@
       <c r="N224" s="3" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="225" spans="1:60" x14ac:dyDescent="0.4">
+      <c r="BM224" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="225" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A225" s="2">
         <f>HEX2DEC(D225)</f>
         <v>269943939</v>
@@ -31023,7 +31153,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="226" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="226" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A226" s="2">
         <f>HEX2DEC(D226)</f>
         <v>269944071</v>
@@ -31067,8 +31197,11 @@
       <c r="N226" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="227" spans="1:60" x14ac:dyDescent="0.4">
+      <c r="BM226" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="227" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A227" s="2">
         <f>HEX2DEC(D227)</f>
         <v>269944577</v>
@@ -31113,7 +31246,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="228" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="228" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A228" s="2">
         <f>HEX2DEC(D228)</f>
         <v>269944579</v>
@@ -31158,7 +31291,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="229" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="229" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A229" s="2">
         <f>HEX2DEC(D229)</f>
         <v>269944843</v>
@@ -31203,7 +31336,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="230" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="230" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A230" s="2">
         <f>HEX2DEC(D230)</f>
         <v>269946624</v>
@@ -31248,7 +31381,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="231" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="231" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A231" s="2">
         <f>HEX2DEC(D231)</f>
         <v>269959937</v>
@@ -31293,7 +31426,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="232" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A232" s="2">
         <f>HEX2DEC(D232)</f>
         <v>269959938</v>
@@ -31338,7 +31471,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="233" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="233" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A233" s="2">
         <f>HEX2DEC(D233)</f>
         <v>269960705</v>
@@ -31383,7 +31516,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="234" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="234" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A234" s="2">
         <f>HEX2DEC(D234)</f>
         <v>269960706</v>
@@ -31428,7 +31561,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="235" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="235" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A235" s="2">
         <f>HEX2DEC(D235)</f>
         <v>270009601</v>
@@ -31485,7 +31618,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="236" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A236" s="2">
         <f>HEX2DEC(D236)</f>
         <v>270017025</v>
@@ -31530,7 +31663,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="237" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="237" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A237" s="2">
         <f>HEX2DEC(D237)</f>
         <v>270017026</v>
@@ -31575,7 +31708,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="238" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A238" s="2">
         <f>HEX2DEC(D238)</f>
         <v>270017281</v>
@@ -31620,7 +31753,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="239" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="239" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A239" s="2">
         <f>HEX2DEC(D239)</f>
         <v>270017537</v>
@@ -31674,7 +31807,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="240" spans="1:60" x14ac:dyDescent="0.4">
+    <row r="240" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A240" s="2">
         <f>HEX2DEC(D240)</f>
         <v>270074113</v>
@@ -31734,8 +31867,11 @@
       <c r="AU240" s="3" t="s">
         <v>2791</v>
       </c>
-    </row>
-    <row r="241" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK240" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="241" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A241" s="2">
         <f>HEX2DEC(D241)</f>
         <v>270074369</v>
@@ -31793,7 +31929,7 @@
         <v>2791</v>
       </c>
     </row>
-    <row r="242" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="242" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A242" s="2">
         <f>HEX2DEC(D242)</f>
         <v>270074625</v>
@@ -31855,8 +31991,11 @@
       <c r="BJ242" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="243" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK242" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="243" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A243" s="2">
         <f>HEX2DEC(D243)</f>
         <v>270074882</v>
@@ -31921,8 +32060,11 @@
       <c r="BJ243" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="244" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK243" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="244" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A244" s="2">
         <f>HEX2DEC(D244)</f>
         <v>270075392</v>
@@ -31984,8 +32126,11 @@
       <c r="BJ244" s="3" t="s">
         <v>2842</v>
       </c>
-    </row>
-    <row r="245" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK244" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="245" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A245" s="2">
         <f>HEX2DEC(D245)</f>
         <v>270139648</v>
@@ -32041,8 +32186,11 @@
       <c r="AU245" s="3" t="s">
         <v>2791</v>
       </c>
-    </row>
-    <row r="246" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK245" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="246" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A246" s="2">
         <f>HEX2DEC(D246)</f>
         <v>270139904</v>
@@ -32106,8 +32254,11 @@
       <c r="BJ246" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="247" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK246" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="247" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A247" s="2">
         <f>HEX2DEC(D247)</f>
         <v>270140161</v>
@@ -32161,7 +32312,7 @@
         <v>2841</v>
       </c>
     </row>
-    <row r="248" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="248" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A248" s="2">
         <f>HEX2DEC(D248)</f>
         <v>270140416</v>
@@ -32226,8 +32377,11 @@
       <c r="BJ248" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="249" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK248" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="249" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A249" s="2">
         <f>HEX2DEC(D249)</f>
         <v>270205184</v>
@@ -32278,7 +32432,7 @@
         <v>2791</v>
       </c>
     </row>
-    <row r="250" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="250" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A250" s="2">
         <f>HEX2DEC(D250)</f>
         <v>270665473</v>
@@ -32374,7 +32528,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="251" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="251" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A251" s="2">
         <f>HEX2DEC(D251)</f>
         <v>270665475</v>
@@ -32470,7 +32624,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="252" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="252" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A252" s="2">
         <f>HEX2DEC(D252)</f>
         <v>270796803</v>
@@ -32569,7 +32723,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="253" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="253" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A253" s="2">
         <f>HEX2DEC(D253)</f>
         <v>270870529</v>
@@ -32668,7 +32822,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="254" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="254" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A254" s="2">
         <f>HEX2DEC(D254)</f>
         <v>270927873</v>
@@ -32713,7 +32867,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="255" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="255" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A255" s="2">
         <f>HEX2DEC(D255)</f>
         <v>270992139</v>
@@ -32758,7 +32912,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="256" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="256" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A256" s="2">
         <f>HEX2DEC(D256)</f>
         <v>271713537</v>
@@ -43192,7 +43346,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="369" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="369" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A369" s="2">
         <f>HEX2DEC(D369)</f>
         <v>538051591</v>
@@ -43294,7 +43448,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="370" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="370" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A370" s="2">
         <f>HEX2DEC(D370)</f>
         <v>538051592</v>
@@ -43396,7 +43550,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="371" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="371" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A371" s="2">
         <f>HEX2DEC(D371)</f>
         <v>538051593</v>
@@ -43498,7 +43652,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="372" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="372" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A372" s="2">
         <f>HEX2DEC(D372)</f>
         <v>538051594</v>
@@ -43600,7 +43754,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="373" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="373" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A373" s="2">
         <f>HEX2DEC(D373)</f>
         <v>538051601</v>
@@ -43702,7 +43856,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="374" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="374" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A374" s="2">
         <f>HEX2DEC(D374)</f>
         <v>538051602</v>
@@ -43804,7 +43958,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="375" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="375" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A375" s="2">
         <f>HEX2DEC(D375)</f>
         <v>538051605</v>
@@ -43906,7 +44060,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="376" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="376" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A376" s="2">
         <f>HEX2DEC(D376)</f>
         <v>538051606</v>
@@ -44008,7 +44162,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="377" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="377" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A377" s="2">
         <f>HEX2DEC(D377)</f>
         <v>538051607</v>
@@ -44110,7 +44264,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="378" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="378" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A378" s="2">
         <f>HEX2DEC(D378)</f>
         <v>538051608</v>
@@ -44212,7 +44366,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="379" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="379" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A379" s="2">
         <f>HEX2DEC(D379)</f>
         <v>538051609</v>
@@ -44314,7 +44468,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="380" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="380" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A380" s="2">
         <f>HEX2DEC(D380)</f>
         <v>538051610</v>
@@ -44416,7 +44570,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="381" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="381" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A381" s="2">
         <f>HEX2DEC(D381)</f>
         <v>538051617</v>
@@ -44518,7 +44672,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="382" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="382" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A382" s="2">
         <f>HEX2DEC(D382)</f>
         <v>538051618</v>
@@ -44619,8 +44773,11 @@
       <c r="AI382" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="383" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BL382" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="383" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A383" s="2">
         <f>HEX2DEC(D383)</f>
         <v>538051619</v>
@@ -44722,7 +44879,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="384" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="384" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A384" s="2">
         <f>HEX2DEC(D384)</f>
         <v>538051620</v>
@@ -49984,7 +50141,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="433" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="433" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A433" s="2">
         <f>HEX2DEC(D433)</f>
         <v>538052875</v>
@@ -50092,7 +50249,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="434" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="434" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A434" s="2">
         <f>HEX2DEC(D434)</f>
         <v>538052876</v>
@@ -50200,7 +50357,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="435" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="435" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A435" s="2">
         <f>HEX2DEC(D435)</f>
         <v>538052877</v>
@@ -50308,7 +50465,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="436" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="436" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A436" s="2">
         <f>HEX2DEC(D436)</f>
         <v>538052878</v>
@@ -50416,7 +50573,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="437" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="437" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A437" s="2">
         <f>HEX2DEC(D437)</f>
         <v>538052879</v>
@@ -50524,7 +50681,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="438" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="438" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A438" s="2">
         <f>HEX2DEC(D438)</f>
         <v>538052880</v>
@@ -50632,7 +50789,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="439" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="439" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A439" s="2">
         <f>HEX2DEC(D439)</f>
         <v>538052881</v>
@@ -50740,7 +50897,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="440" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="440" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A440" s="2">
         <f>HEX2DEC(D440)</f>
         <v>538052882</v>
@@ -50848,7 +51005,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="441" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="441" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A441" s="2">
         <f>HEX2DEC(D441)</f>
         <v>538052883</v>
@@ -50956,7 +51113,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="442" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="442" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A442" s="2">
         <f>HEX2DEC(D442)</f>
         <v>538053121</v>
@@ -51063,8 +51220,11 @@
       <c r="AI442" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="443" spans="1:35" x14ac:dyDescent="0.4">
+      <c r="BL442" s="3" t="s">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="443" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A443" s="2">
         <f>HEX2DEC(D443)</f>
         <v>538053633</v>
@@ -51166,7 +51326,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="444" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="444" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A444" s="2">
         <f>HEX2DEC(D444)</f>
         <v>538053634</v>
@@ -51268,7 +51428,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="445" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="445" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A445" s="2">
         <f>HEX2DEC(D445)</f>
         <v>538053636</v>
@@ -51370,7 +51530,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="446" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="446" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A446" s="2">
         <f>HEX2DEC(D446)</f>
         <v>538053639</v>
@@ -51472,7 +51632,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="447" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="447" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A447" s="2">
         <f>HEX2DEC(D447)</f>
         <v>538053643</v>
@@ -51575,7 +51735,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="448" spans="1:35" x14ac:dyDescent="0.4">
+    <row r="448" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A448" s="2">
         <f>HEX2DEC(D448)</f>
         <v>538055434</v>
@@ -51677,7 +51837,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="449" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="449" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A449" s="2">
         <f>HEX2DEC(D449)</f>
         <v>538055941</v>
@@ -51779,7 +51939,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="450" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="450" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A450" s="2">
         <f>HEX2DEC(D450)</f>
         <v>538055942</v>
@@ -51881,7 +52041,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="451" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="451" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A451" s="2">
         <f>HEX2DEC(D451)</f>
         <v>538056709</v>
@@ -51904,8 +52064,8 @@
       <c r="G451" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H451" s="1" t="s">
-        <v>86</v>
+      <c r="H451" s="3" t="s">
+        <v>2853</v>
       </c>
       <c r="I451" s="1" t="s">
         <v>43</v>
@@ -51988,8 +52148,9 @@
       <c r="AI451" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="452" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK451" s="5"/>
+    </row>
+    <row r="452" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A452" s="2">
         <f>HEX2DEC(D452)</f>
         <v>538056969</v>
@@ -52096,8 +52257,9 @@
       <c r="AI452" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="453" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK452" s="5"/>
+    </row>
+    <row r="453" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A453" s="2">
         <f>HEX2DEC(D453)</f>
         <v>538057731</v>
@@ -52198,8 +52360,9 @@
       <c r="AI453" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="454" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK453" s="5"/>
+    </row>
+    <row r="454" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A454" s="2">
         <f>HEX2DEC(D454)</f>
         <v>538069761</v>
@@ -52309,8 +52472,9 @@
       <c r="AY454" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="455" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK454" s="5"/>
+    </row>
+    <row r="455" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A455" s="2">
         <f>HEX2DEC(D455)</f>
         <v>538069762</v>
@@ -52420,8 +52584,9 @@
       <c r="AY455" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="456" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK455" s="5"/>
+    </row>
+    <row r="456" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A456" s="2">
         <f>HEX2DEC(D456)</f>
         <v>538069763</v>
@@ -52531,8 +52696,12 @@
       <c r="AY456" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="457" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK456" s="5"/>
+      <c r="BL456" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="457" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A457" s="2">
         <f>HEX2DEC(D457)</f>
         <v>538069764</v>
@@ -52668,8 +52837,9 @@
       <c r="BH457" s="5"/>
       <c r="BI457" s="5"/>
       <c r="BJ457" s="5"/>
-    </row>
-    <row r="458" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK457" s="5"/>
+    </row>
+    <row r="458" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A458" s="2">
         <f>HEX2DEC(D458)</f>
         <v>538069768</v>
@@ -52805,8 +52975,12 @@
       <c r="BH458" s="5"/>
       <c r="BI458" s="5"/>
       <c r="BJ458" s="5"/>
-    </row>
-    <row r="459" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK458" s="5"/>
+      <c r="BL458" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="459" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A459" s="2">
         <f>HEX2DEC(D459)</f>
         <v>538116353</v>
@@ -52938,8 +53112,9 @@
       <c r="BH459" s="5"/>
       <c r="BI459" s="5"/>
       <c r="BJ459" s="5"/>
-    </row>
-    <row r="460" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK459" s="5"/>
+    </row>
+    <row r="460" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A460" s="2">
         <f>HEX2DEC(D460)</f>
         <v>538116354</v>
@@ -53071,8 +53246,9 @@
       <c r="BH460" s="5"/>
       <c r="BI460" s="5"/>
       <c r="BJ460" s="5"/>
-    </row>
-    <row r="461" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BK460" s="5"/>
+    </row>
+    <row r="461" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A461" s="2">
         <f>HEX2DEC(D461)</f>
         <v>538116609</v>
@@ -53175,7 +53351,7 @@
       </c>
       <c r="XFD461" s="4"/>
     </row>
-    <row r="462" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="462" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A462" s="2">
         <f>HEX2DEC(D462)</f>
         <v>538116610</v>
@@ -53281,7 +53457,7 @@
       </c>
       <c r="XFD462" s="4"/>
     </row>
-    <row r="463" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="463" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A463" s="2">
         <f>HEX2DEC(D463)</f>
         <v>538116613</v>
@@ -53387,7 +53563,7 @@
       </c>
       <c r="XFD463" s="4"/>
     </row>
-    <row r="464" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="464" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A464" s="2">
         <f>HEX2DEC(D464)</f>
         <v>538116865</v>
@@ -53490,7 +53666,7 @@
       </c>
       <c r="XFD464" s="4"/>
     </row>
-    <row r="465" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="465" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A465" s="2">
         <f>HEX2DEC(D465)</f>
         <v>538116866</v>
@@ -53593,7 +53769,7 @@
       </c>
       <c r="XFD465" s="4"/>
     </row>
-    <row r="466" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="466" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A466" s="2">
         <f>HEX2DEC(D466)</f>
         <v>538116867</v>
@@ -53696,7 +53872,7 @@
       </c>
       <c r="XFD466" s="4"/>
     </row>
-    <row r="467" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="467" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A467" s="2">
         <f>HEX2DEC(D467)</f>
         <v>538116868</v>
@@ -53799,7 +53975,7 @@
       </c>
       <c r="XFD467" s="4"/>
     </row>
-    <row r="468" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="468" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A468" s="2">
         <f>HEX2DEC(D468)</f>
         <v>538116869</v>
@@ -53902,7 +54078,7 @@
       </c>
       <c r="XFD468" s="4"/>
     </row>
-    <row r="469" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="469" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A469" s="2">
         <f>HEX2DEC(D469)</f>
         <v>538116870</v>
@@ -54008,7 +54184,7 @@
       </c>
       <c r="XFD469" s="4"/>
     </row>
-    <row r="470" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="470" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A470" s="2">
         <f>HEX2DEC(D470)</f>
         <v>538117121</v>
@@ -54112,7 +54288,7 @@
       </c>
       <c r="XFD470" s="4"/>
     </row>
-    <row r="471" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="471" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A471" s="2">
         <f>HEX2DEC(D471)</f>
         <v>538117122</v>
@@ -54216,7 +54392,7 @@
       </c>
       <c r="XFD471" s="4"/>
     </row>
-    <row r="472" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="472" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A472" s="2">
         <f>HEX2DEC(D472)</f>
         <v>538117123</v>
@@ -54320,7 +54496,7 @@
       </c>
       <c r="XFD472" s="4"/>
     </row>
-    <row r="473" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="473" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A473" s="2">
         <f>HEX2DEC(D473)</f>
         <v>538117377</v>
@@ -54417,7 +54593,7 @@
       </c>
       <c r="XFD473" s="4"/>
     </row>
-    <row r="474" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="474" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A474" s="2">
         <f>HEX2DEC(D474)</f>
         <v>538117889</v>
@@ -54515,9 +54691,12 @@
       <c r="AI474" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="BK474" s="6" t="s">
+        <v>2846</v>
+      </c>
       <c r="XFD474" s="4"/>
     </row>
-    <row r="475" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="475" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A475" s="2">
         <f>HEX2DEC(D475)</f>
         <v>538120705</v>
@@ -54621,9 +54800,10 @@
       <c r="AI475" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="BK475" s="6"/>
       <c r="XFD475" s="4"/>
     </row>
-    <row r="476" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="476" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A476" s="2">
         <f>HEX2DEC(D476)</f>
         <v>538120706</v>
@@ -54727,9 +54907,10 @@
       <c r="AI476" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="BK476" s="6"/>
       <c r="XFD476" s="4"/>
     </row>
-    <row r="477" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="477" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A477" s="2">
         <f>HEX2DEC(D477)</f>
         <v>538124803</v>
@@ -54841,7 +55022,7 @@
       </c>
       <c r="XFD477" s="4"/>
     </row>
-    <row r="478" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="478" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A478" s="2">
         <f>HEX2DEC(D478)</f>
         <v>538124804</v>
@@ -54951,9 +55132,10 @@
       <c r="BE478" s="6" t="s">
         <v>2808</v>
       </c>
+      <c r="BK478" s="1"/>
       <c r="XFD478" s="4"/>
     </row>
-    <row r="479" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="479" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A479" s="2">
         <f>HEX2DEC(D479)</f>
         <v>538134017</v>
@@ -55060,9 +55242,12 @@
       <c r="BJ479" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK479" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD479" s="4"/>
     </row>
-    <row r="480" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="480" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A480" s="2">
         <f>HEX2DEC(D480)</f>
         <v>538134018</v>
@@ -55169,9 +55354,12 @@
       <c r="BJ480" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK480" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD480" s="4"/>
     </row>
-    <row r="481" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="481" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A481" s="2">
         <f>HEX2DEC(D481)</f>
         <v>538134019</v>
@@ -55278,9 +55466,12 @@
       <c r="BJ481" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK481" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD481" s="4"/>
     </row>
-    <row r="482" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="482" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A482" s="2">
         <f>HEX2DEC(D482)</f>
         <v>538134020</v>
@@ -55387,9 +55578,12 @@
       <c r="BJ482" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK482" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD482" s="4"/>
     </row>
-    <row r="483" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="483" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A483" s="2">
         <f>HEX2DEC(D483)</f>
         <v>538137089</v>
@@ -55490,9 +55684,10 @@
       <c r="AQ483" s="6" t="s">
         <v>2791</v>
       </c>
+      <c r="BK483" s="1"/>
       <c r="XFD483" s="4"/>
     </row>
-    <row r="484" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="484" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A484" s="2">
         <f>HEX2DEC(D484)</f>
         <v>538137090</v>
@@ -55619,9 +55814,10 @@
       <c r="BH484" s="1"/>
       <c r="BI484" s="1"/>
       <c r="BJ484" s="1"/>
+      <c r="BK484" s="1"/>
       <c r="XFD484" s="4"/>
     </row>
-    <row r="485" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="485" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A485" s="2">
         <f>HEX2DEC(D485)</f>
         <v>538137347</v>
@@ -55750,9 +55946,10 @@
       <c r="BH485" s="1"/>
       <c r="BI485" s="1"/>
       <c r="BJ485" s="1"/>
+      <c r="BK485" s="1"/>
       <c r="XFD485" s="4"/>
     </row>
-    <row r="486" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="486" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A486" s="2">
         <f>HEX2DEC(D486)</f>
         <v>538181889</v>
@@ -55882,9 +56079,10 @@
       <c r="BH486" s="1"/>
       <c r="BI486" s="1"/>
       <c r="BJ486" s="1"/>
+      <c r="BK486" s="1"/>
       <c r="XFD486" s="4"/>
     </row>
-    <row r="487" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="487" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A487" s="2">
         <f>HEX2DEC(D487)</f>
         <v>538181890</v>
@@ -56014,9 +56212,10 @@
       <c r="BH487" s="1"/>
       <c r="BI487" s="1"/>
       <c r="BJ487" s="1"/>
+      <c r="BK487" s="1"/>
       <c r="XFD487" s="4"/>
     </row>
-    <row r="488" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="488" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A488" s="2">
         <f>HEX2DEC(D488)</f>
         <v>538182145</v>
@@ -56118,7 +56317,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="489" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="489" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A489" s="2">
         <f>HEX2DEC(D489)</f>
         <v>538182146</v>
@@ -56220,7 +56419,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="490" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="490" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A490" s="2">
         <f>HEX2DEC(D490)</f>
         <v>538182401</v>
@@ -56322,7 +56521,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="491" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="491" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A491" s="2">
         <f>HEX2DEC(D491)</f>
         <v>538182402</v>
@@ -56424,7 +56623,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="492" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="492" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A492" s="2">
         <f>HEX2DEC(D492)</f>
         <v>538182403</v>
@@ -56526,7 +56725,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="493" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="493" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A493" s="2">
         <f>HEX2DEC(D493)</f>
         <v>538182404</v>
@@ -56628,7 +56827,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="494" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="494" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A494" s="2">
         <f>HEX2DEC(D494)</f>
         <v>538182657</v>
@@ -56730,7 +56929,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="495" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="495" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A495" s="2">
         <f>HEX2DEC(D495)</f>
         <v>538182658</v>
@@ -56832,7 +57031,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="496" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="496" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A496" s="2">
         <f>HEX2DEC(D496)</f>
         <v>538182659</v>
@@ -58560,7 +58759,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="513" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="513" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A513" s="2">
         <f>HEX2DEC(D513)</f>
         <v>538264066</v>
@@ -58659,7 +58858,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="514" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="514" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A514" s="2">
         <f>HEX2DEC(D514)</f>
         <v>538280961</v>
@@ -58764,8 +58963,11 @@
         <v>2791</v>
       </c>
       <c r="AS514" s="3"/>
-    </row>
-    <row r="515" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="BK514" s="3" t="s">
+        <v>2846</v>
+      </c>
+    </row>
+    <row r="515" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A515" s="2">
         <f>HEX2DEC(D515)</f>
         <v>538280962</v>
@@ -58870,8 +59072,11 @@
         <v>2791</v>
       </c>
       <c r="AS515" s="3"/>
-    </row>
-    <row r="516" spans="1:45" x14ac:dyDescent="0.4">
+      <c r="BK515" s="3" t="s">
+        <v>2846</v>
+      </c>
+    </row>
+    <row r="516" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A516" s="2">
         <f>HEX2DEC(D516)</f>
         <v>538312961</v>
@@ -58916,7 +59121,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="517" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="517" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A517" s="2">
         <f>HEX2DEC(D517)</f>
         <v>538312977</v>
@@ -58961,7 +59166,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="518" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="518" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A518" s="2">
         <f>HEX2DEC(D518)</f>
         <v>538313217</v>
@@ -59006,7 +59211,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="519" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="519" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A519" s="2">
         <f>HEX2DEC(D519)</f>
         <v>538313233</v>
@@ -59051,7 +59256,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="520" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="520" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A520" s="2">
         <f>HEX2DEC(D520)</f>
         <v>538313473</v>
@@ -59096,7 +59301,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="521" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="521" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A521" s="2">
         <f>HEX2DEC(D521)</f>
         <v>538313474</v>
@@ -59141,7 +59346,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="522" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="522" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A522" s="2">
         <f>HEX2DEC(D522)</f>
         <v>538313729</v>
@@ -59186,7 +59391,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="523" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="523" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A523" s="2">
         <f>HEX2DEC(D523)</f>
         <v>538313730</v>
@@ -59231,7 +59436,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="524" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="524" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A524" s="2">
         <f>HEX2DEC(D524)</f>
         <v>538313731</v>
@@ -59276,7 +59481,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="525" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="525" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A525" s="2">
         <f>HEX2DEC(D525)</f>
         <v>538317057</v>
@@ -59375,7 +59580,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="526" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="526" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A526" s="2">
         <f>HEX2DEC(D526)</f>
         <v>538317313</v>
@@ -59477,7 +59682,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="527" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="527" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A527" s="2">
         <f>HEX2DEC(D527)</f>
         <v>538317569</v>
@@ -59582,7 +59787,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="528" spans="1:45" x14ac:dyDescent="0.4">
+    <row r="528" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A528" s="2">
         <f>HEX2DEC(D528)</f>
         <v>538317825</v>
@@ -59687,7 +59892,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="529" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="529" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A529" s="2">
         <f>HEX2DEC(D529)</f>
         <v>538317826</v>
@@ -59792,7 +59997,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="530" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="530" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A530" s="2">
         <f>HEX2DEC(D530)</f>
         <v>538318081</v>
@@ -59897,7 +60102,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="531" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="531" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A531" s="2">
         <f>HEX2DEC(D531)</f>
         <v>538318082</v>
@@ -60002,7 +60207,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="532" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="532" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A532" s="2">
         <f>HEX2DEC(D532)</f>
         <v>538318337</v>
@@ -60107,7 +60312,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="533" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="533" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A533" s="2">
         <f>HEX2DEC(D533)</f>
         <v>538318338</v>
@@ -60212,7 +60417,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="534" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="534" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A534" s="2">
         <f>HEX2DEC(D534)</f>
         <v>538326785</v>
@@ -60329,7 +60534,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="535" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="535" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A535" s="2">
         <f>HEX2DEC(D535)</f>
         <v>538326786</v>
@@ -60449,7 +60654,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="536" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="536" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A536" s="2">
         <f>HEX2DEC(D536)</f>
         <v>538326788</v>
@@ -60569,7 +60774,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="537" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="537" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A537" s="2">
         <f>HEX2DEC(D537)</f>
         <v>538330369</v>
@@ -60613,8 +60818,11 @@
       <c r="N537" s="3" t="s">
         <v>1099</v>
       </c>
-    </row>
-    <row r="538" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BK537" s="3" t="s">
+        <v>2846</v>
+      </c>
+    </row>
+    <row r="538" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A538" s="2">
         <f>HEX2DEC(D538)</f>
         <v>538378497</v>
@@ -60659,7 +60867,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="539" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="539" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A539" s="2">
         <f>HEX2DEC(D539)</f>
         <v>538379281</v>
@@ -60703,8 +60911,11 @@
       <c r="N539" s="3" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="540" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BM539" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="540" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A540" s="2">
         <f>HEX2DEC(D540)</f>
         <v>538379330</v>
@@ -60748,8 +60959,11 @@
       <c r="N540" s="3" t="s">
         <v>1099</v>
       </c>
-    </row>
-    <row r="541" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BM540" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="541" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A541" s="2">
         <f>HEX2DEC(D541)</f>
         <v>538379527</v>
@@ -60793,8 +61007,11 @@
       <c r="N541" s="3" t="s">
         <v>1099</v>
       </c>
-    </row>
-    <row r="542" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BM541" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="542" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A542" s="2">
         <f>HEX2DEC(D542)</f>
         <v>538380033</v>
@@ -60839,7 +61056,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="543" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="543" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A543" s="2">
         <f>HEX2DEC(D543)</f>
         <v>538380035</v>
@@ -60884,7 +61101,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="544" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="544" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A544" s="2">
         <f>HEX2DEC(D544)</f>
         <v>538382080</v>
@@ -60929,7 +61146,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="545" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="545" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A545" s="2">
         <f>HEX2DEC(D545)</f>
         <v>538395138</v>
@@ -60974,7 +61191,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="546" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="546" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A546" s="2">
         <f>HEX2DEC(D546)</f>
         <v>538395393</v>
@@ -61019,7 +61236,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="547" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="547" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A547" s="2">
         <f>HEX2DEC(D547)</f>
         <v>538395394</v>
@@ -61064,7 +61281,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="548" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="548" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A548" s="2">
         <f>HEX2DEC(D548)</f>
         <v>538395651</v>
@@ -61109,7 +61326,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="549" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="549" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A549" s="2">
         <f>HEX2DEC(D549)</f>
         <v>538395655</v>
@@ -61154,7 +61371,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="550" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="550" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A550" s="2">
         <f>HEX2DEC(D550)</f>
         <v>538395779</v>
@@ -61198,8 +61415,11 @@
       <c r="N550" s="3" t="s">
         <v>1858</v>
       </c>
-    </row>
-    <row r="551" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BM550" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="551" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A551" s="2">
         <f>HEX2DEC(D551)</f>
         <v>538396161</v>
@@ -61244,7 +61464,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="552" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="552" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A552" s="2">
         <f>HEX2DEC(D552)</f>
         <v>538396162</v>
@@ -61289,7 +61509,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="553" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="553" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A553" s="2">
         <f>HEX2DEC(D553)</f>
         <v>538444033</v>
@@ -61334,7 +61554,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="554" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="554" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A554" s="2">
         <f>HEX2DEC(D554)</f>
         <v>538445057</v>
@@ -61386,7 +61606,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="555" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="555" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A555" s="2">
         <f>HEX2DEC(D555)</f>
         <v>538452737</v>
@@ -61431,7 +61651,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="556" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="556" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A556" s="2">
         <f>HEX2DEC(D556)</f>
         <v>538452993</v>
@@ -61488,7 +61708,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="557" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="557" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A557" s="2">
         <f>HEX2DEC(D557)</f>
         <v>538509569</v>
@@ -61557,8 +61777,11 @@
       <c r="BC557" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="558" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK557" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="558" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A558" s="2">
         <f>HEX2DEC(D558)</f>
         <v>538510081</v>
@@ -61632,8 +61855,11 @@
       <c r="BJ558" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="559" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK558" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="559" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A559" s="2">
         <f>HEX2DEC(D559)</f>
         <v>538510338</v>
@@ -61707,8 +61933,11 @@
       <c r="BJ559" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="560" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK559" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="560" spans="1:65" x14ac:dyDescent="0.4">
       <c r="A560" s="2">
         <f>HEX2DEC(D560)</f>
         <v>538510848</v>
@@ -61773,8 +62002,11 @@
       <c r="BJ560" s="3" t="s">
         <v>2842</v>
       </c>
-    </row>
-    <row r="561" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK560" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="561" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A561" s="2">
         <f>HEX2DEC(D561)</f>
         <v>538575104</v>
@@ -61833,8 +62065,11 @@
       <c r="AU561" s="3" t="s">
         <v>2791</v>
       </c>
-    </row>
-    <row r="562" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK561" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="562" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A562" s="2">
         <f>HEX2DEC(D562)</f>
         <v>538575360</v>
@@ -61914,8 +62149,11 @@
       <c r="BJ562" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="563" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK562" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="563" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A563" s="2">
         <f>HEX2DEC(D563)</f>
         <v>538575617</v>
@@ -61971,8 +62209,11 @@
       <c r="BJ563" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="564" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK563" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="564" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A564" s="2">
         <f>HEX2DEC(D564)</f>
         <v>538575872</v>
@@ -62040,8 +62281,11 @@
       <c r="BJ564" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="565" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK564" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="565" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A565" s="2">
         <f>HEX2DEC(D565)</f>
         <v>538640640</v>
@@ -62093,7 +62337,7 @@
       </c>
       <c r="AV565" s="3"/>
     </row>
-    <row r="566" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="566" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A566" s="2">
         <f>HEX2DEC(D566)</f>
         <v>538640898</v>
@@ -62144,7 +62388,7 @@
         <v>2791</v>
       </c>
     </row>
-    <row r="567" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="567" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A567" s="2">
         <f>HEX2DEC(D567)</f>
         <v>539100929</v>
@@ -62243,7 +62487,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="568" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="568" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A568" s="2">
         <f>HEX2DEC(D568)</f>
         <v>539100931</v>
@@ -62342,7 +62586,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="569" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="569" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A569" s="2">
         <f>HEX2DEC(D569)</f>
         <v>539232259</v>
@@ -62444,7 +62688,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="570" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="570" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A570" s="2">
         <f>HEX2DEC(D570)</f>
         <v>539305985</v>
@@ -62546,7 +62790,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="571" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="571" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A571" s="2">
         <f>HEX2DEC(D571)</f>
         <v>539363329</v>
@@ -62591,7 +62835,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="572" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="572" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A572" s="2">
         <f>HEX2DEC(D572)</f>
         <v>539427595</v>
@@ -62636,7 +62880,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="573" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="573" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A573" s="2">
         <f>HEX2DEC(D573)</f>
         <v>540148993</v>
@@ -62732,7 +62976,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="574" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="574" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A574" s="2">
         <f>HEX2DEC(D574)</f>
         <v>540148994</v>
@@ -62828,7 +63072,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="575" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="575" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A575" s="2">
         <f>HEX2DEC(D575)</f>
         <v>540148995</v>
@@ -62924,7 +63168,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="576" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="576" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A576" s="2">
         <f>HEX2DEC(D576)</f>
         <v>540148996</v>
@@ -68631,7 +68875,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="641" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="641" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A641" s="2">
         <f>HEX2DEC(D641)</f>
         <v>555095554</v>
@@ -68736,7 +68980,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="642" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="642" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A642" s="2">
         <f>HEX2DEC(D642)</f>
         <v>556205828</v>
@@ -68787,7 +69031,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="643" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="643" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A643" s="2">
         <f>HEX2DEC(D643)</f>
         <v>556205834</v>
@@ -68838,7 +69082,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="644" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="644" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A644" s="2">
         <f>HEX2DEC(D644)</f>
         <v>562203136</v>
@@ -68937,7 +69181,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="645" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="645" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A645" s="2">
         <f>HEX2DEC(D645)</f>
         <v>571934980</v>
@@ -68985,7 +69229,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="646" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="646" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A646" s="2">
         <f>HEX2DEC(D646)</f>
         <v>571934986</v>
@@ -69033,7 +69277,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="647" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="647" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A647" s="2">
         <f>HEX2DEC(D647)</f>
         <v>574752768</v>
@@ -69144,7 +69388,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="648" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="648" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A648" s="2">
         <f>HEX2DEC(D648)</f>
         <v>574948865</v>
@@ -69240,7 +69484,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="649" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="649" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A649" s="2">
         <f>HEX2DEC(D649)</f>
         <v>722601996</v>
@@ -69341,8 +69585,11 @@
       <c r="AI649" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="650" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL649" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="650" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A650" s="2">
         <f>HEX2DEC(D650)</f>
         <v>722601997</v>
@@ -69443,8 +69690,11 @@
       <c r="AI650" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="651" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL650" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="651" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A651" s="2">
         <f>HEX2DEC(D651)</f>
         <v>756176910</v>
@@ -69550,7 +69800,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="652" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="652" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A652" s="2">
         <f>HEX2DEC(D652)</f>
         <v>756181003</v>
@@ -69656,7 +69906,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="653" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="653" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A653" s="2">
         <f>HEX2DEC(D653)</f>
         <v>806421772</v>
@@ -69761,8 +70011,11 @@
       <c r="AI653" s="1" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="654" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL653" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="654" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A654" s="2">
         <f>HEX2DEC(D654)</f>
         <v>806487041</v>
@@ -69864,8 +70117,11 @@
       <c r="AI654" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="655" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL654" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="655" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A655" s="2">
         <f>HEX2DEC(D655)</f>
         <v>806487045</v>
@@ -69968,7 +70224,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="656" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="656" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A656" s="2">
         <f>HEX2DEC(D656)</f>
         <v>806487057</v>
@@ -70076,7 +70332,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="657" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="657" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A657" s="2">
         <f>HEX2DEC(D657)</f>
         <v>806487058</v>
@@ -70184,7 +70440,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="658" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="658" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A658" s="2">
         <f>HEX2DEC(D658)</f>
         <v>806487061</v>
@@ -70292,7 +70548,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="659" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="659" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A659" s="2">
         <f>HEX2DEC(D659)</f>
         <v>806487064</v>
@@ -70400,7 +70656,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="660" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="660" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A660" s="2">
         <f>HEX2DEC(D660)</f>
         <v>806487066</v>
@@ -70507,8 +70763,11 @@
       <c r="AI660" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="661" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL660" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="661" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A661" s="2">
         <f>HEX2DEC(D661)</f>
         <v>806487073</v>
@@ -70616,7 +70875,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="662" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="662" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A662" s="2">
         <f>HEX2DEC(D662)</f>
         <v>806487297</v>
@@ -70724,7 +70983,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="663" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="663" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A663" s="2">
         <f>HEX2DEC(D663)</f>
         <v>806487554</v>
@@ -70832,7 +71091,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="664" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="664" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A664" s="2">
         <f>HEX2DEC(D664)</f>
         <v>806487556</v>
@@ -70940,7 +71199,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="665" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="665" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A665" s="2">
         <f>HEX2DEC(D665)</f>
         <v>806487809</v>
@@ -71048,7 +71307,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="666" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="666" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A666" s="2">
         <f>HEX2DEC(D666)</f>
         <v>806488083</v>
@@ -71156,7 +71415,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="667" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="667" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A667" s="2">
         <f>HEX2DEC(D667)</f>
         <v>806490881</v>
@@ -71261,7 +71520,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="668" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="668" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A668" s="2">
         <f>HEX2DEC(D668)</f>
         <v>806490882</v>
@@ -71366,7 +71625,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="669" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="669" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A669" s="2">
         <f>HEX2DEC(D669)</f>
         <v>806491138</v>
@@ -71471,8 +71730,11 @@
       <c r="BF669" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="670" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL669" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="670" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A670" s="2">
         <f>HEX2DEC(D670)</f>
         <v>806491140</v>
@@ -71575,7 +71837,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="671" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="671" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A671" s="2">
         <f>HEX2DEC(D671)</f>
         <v>806491396</v>
@@ -71688,8 +71950,11 @@
       <c r="BF671" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="672" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL671" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="672" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A672" s="2">
         <f>HEX2DEC(D672)</f>
         <v>806491651</v>
@@ -71800,7 +72065,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="673" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="673" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A673" s="2">
         <f>HEX2DEC(D673)</f>
         <v>806491653</v>
@@ -71910,8 +72175,11 @@
       <c r="BF673" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="674" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL673" s="3" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="674" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A674" s="2">
         <f>HEX2DEC(D674)</f>
         <v>806491657</v>
@@ -72019,7 +72287,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="675" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="675" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A675" s="2">
         <f>HEX2DEC(D675)</f>
         <v>806495745</v>
@@ -72130,7 +72398,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="676" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="676" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A676" s="2">
         <f>HEX2DEC(D676)</f>
         <v>806495746</v>
@@ -72238,7 +72506,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="677" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="677" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A677" s="2">
         <f>HEX2DEC(D677)</f>
         <v>806499077</v>
@@ -72343,7 +72611,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="678" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="678" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A678" s="2">
         <f>HEX2DEC(D678)</f>
         <v>806499079</v>
@@ -72448,7 +72716,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="679" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="679" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A679" s="2">
         <f>HEX2DEC(D679)</f>
         <v>806499337</v>
@@ -72551,7 +72819,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="680" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="680" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A680" s="2">
         <f>HEX2DEC(D680)</f>
         <v>806499338</v>
@@ -72654,7 +72922,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="681" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="681" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A681" s="2">
         <f>HEX2DEC(D681)</f>
         <v>806499841</v>
@@ -72765,7 +73033,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="682" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="682" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A682" s="2">
         <f>HEX2DEC(D682)</f>
         <v>806500098</v>
@@ -72873,7 +73141,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="683" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="683" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A683" s="2">
         <f>HEX2DEC(D683)</f>
         <v>806500099</v>
@@ -72981,7 +73249,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="684" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="684" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A684" s="2">
         <f>HEX2DEC(D684)</f>
         <v>806500100</v>
@@ -73089,7 +73357,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="685" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="685" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A685" s="2">
         <f>HEX2DEC(D685)</f>
         <v>806500105</v>
@@ -73197,7 +73465,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="686" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="686" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A686" s="2">
         <f>HEX2DEC(D686)</f>
         <v>806500106</v>
@@ -73307,8 +73575,11 @@
       <c r="BF686" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="687" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL686" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="687" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A687" s="2">
         <f>HEX2DEC(D687)</f>
         <v>806504449</v>
@@ -73416,7 +73687,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="688" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="688" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A688" s="2">
         <f>HEX2DEC(D688)</f>
         <v>806504450</v>
@@ -73527,7 +73798,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="689" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="689" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A689" s="2">
         <f>HEX2DEC(D689)</f>
         <v>806504705</v>
@@ -73638,7 +73909,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="690" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="690" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A690" s="2">
         <f>HEX2DEC(D690)</f>
         <v>806504708</v>
@@ -73749,7 +74020,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="691" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="691" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A691" s="2">
         <f>HEX2DEC(D691)</f>
         <v>806504710</v>
@@ -73860,7 +74131,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="692" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="692" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A692" s="2">
         <f>HEX2DEC(D692)</f>
         <v>806504723</v>
@@ -73967,8 +74238,11 @@
       <c r="AI692" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="693" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL692" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="693" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A693" s="2">
         <f>HEX2DEC(D693)</f>
         <v>806505220</v>
@@ -74078,8 +74352,11 @@
       <c r="AY693" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="694" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL693" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="694" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A694" s="2">
         <f>HEX2DEC(D694)</f>
         <v>806507523</v>
@@ -74181,8 +74458,11 @@
       <c r="AI694" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="695" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL694" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="695" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A695" s="2">
         <f>HEX2DEC(D695)</f>
         <v>806508553</v>
@@ -74290,7 +74570,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="696" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="696" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A696" s="2">
         <f>HEX2DEC(D696)</f>
         <v>806508802</v>
@@ -74398,7 +74678,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="697" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="697" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A697" s="2">
         <f>HEX2DEC(D697)</f>
         <v>806508817</v>
@@ -74505,8 +74785,11 @@
       <c r="AI697" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="698" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL697" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="698" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A698" s="2">
         <f>HEX2DEC(D698)</f>
         <v>806512643</v>
@@ -74614,7 +74897,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="699" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="699" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A699" s="2">
         <f>HEX2DEC(D699)</f>
         <v>806512644</v>
@@ -74722,7 +75005,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="700" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="700" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A700" s="2">
         <f>HEX2DEC(D700)</f>
         <v>806512648</v>
@@ -74832,8 +75115,11 @@
       <c r="BF700" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="701" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL700" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="701" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A701" s="2">
         <f>HEX2DEC(D701)</f>
         <v>806512899</v>
@@ -74941,7 +75227,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="702" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="702" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A702" s="2">
         <f>HEX2DEC(D702)</f>
         <v>806512907</v>
@@ -75048,8 +75334,11 @@
       <c r="AI702" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="703" spans="1:58" x14ac:dyDescent="0.4">
+      <c r="BL702" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="703" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A703" s="2">
         <f>HEX2DEC(D703)</f>
         <v>806512909</v>
@@ -75157,7 +75446,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="704" spans="1:58" x14ac:dyDescent="0.4">
+    <row r="704" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A704" s="2">
         <f>HEX2DEC(D704)</f>
         <v>806512910</v>
@@ -75264,8 +75553,9 @@
       <c r="AI704" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="705" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BK704" s="5"/>
+    </row>
+    <row r="705" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A705" s="2">
         <f>HEX2DEC(D705)</f>
         <v>806512912</v>
@@ -75372,9 +75662,12 @@
       <c r="AI705" s="1" t="s">
         <v>116</v>
       </c>
+      <c r="BL705" s="6" t="s">
+        <v>2854</v>
+      </c>
       <c r="XFD705" s="4"/>
     </row>
-    <row r="706" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="706" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A706" s="2">
         <f>HEX2DEC(D706)</f>
         <v>806516741</v>
@@ -75486,7 +75779,7 @@
       </c>
       <c r="XFD706" s="4"/>
     </row>
-    <row r="707" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="707" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A707" s="2">
         <f>HEX2DEC(D707)</f>
         <v>806551809</v>
@@ -75598,7 +75891,7 @@
       </c>
       <c r="XFD707" s="4"/>
     </row>
-    <row r="708" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="708" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A708" s="2">
         <f>HEX2DEC(D708)</f>
         <v>806551810</v>
@@ -75719,7 +76012,7 @@
       </c>
       <c r="XFD708" s="4"/>
     </row>
-    <row r="709" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="709" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A709" s="2">
         <f>HEX2DEC(D709)</f>
         <v>806552325</v>
@@ -75834,7 +76127,7 @@
       </c>
       <c r="XFD709" s="4"/>
     </row>
-    <row r="710" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="710" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A710" s="2">
         <f>HEX2DEC(D710)</f>
         <v>806552577</v>
@@ -75943,7 +76236,7 @@
       </c>
       <c r="XFD710" s="4"/>
     </row>
-    <row r="711" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="711" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A711" s="2">
         <f>HEX2DEC(D711)</f>
         <v>806552578</v>
@@ -76052,7 +76345,7 @@
       </c>
       <c r="XFD711" s="4"/>
     </row>
-    <row r="712" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="712" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A712" s="2">
         <f>HEX2DEC(D712)</f>
         <v>806552579</v>
@@ -76161,7 +76454,7 @@
       </c>
       <c r="XFD712" s="4"/>
     </row>
-    <row r="713" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="713" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A713" s="2">
         <f>HEX2DEC(D713)</f>
         <v>806552833</v>
@@ -76267,7 +76560,7 @@
       </c>
       <c r="XFD713" s="4"/>
     </row>
-    <row r="714" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="714" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A714" s="2">
         <f>HEX2DEC(D714)</f>
         <v>806560259</v>
@@ -76380,7 +76673,7 @@
       </c>
       <c r="XFD714" s="4"/>
     </row>
-    <row r="715" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="715" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A715" s="2">
         <f>HEX2DEC(D715)</f>
         <v>806560260</v>
@@ -76493,7 +76786,7 @@
       </c>
       <c r="XFD715" s="4"/>
     </row>
-    <row r="716" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="716" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A716" s="2">
         <f>HEX2DEC(D716)</f>
         <v>806560261</v>
@@ -76614,7 +76907,7 @@
       </c>
       <c r="XFD716" s="4"/>
     </row>
-    <row r="717" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="717" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A717" s="2">
         <f>HEX2DEC(D717)</f>
         <v>806560518</v>
@@ -76729,7 +77022,7 @@
       </c>
       <c r="XFD717" s="4"/>
     </row>
-    <row r="718" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="718" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A718" s="2">
         <f>HEX2DEC(D718)</f>
         <v>806568449</v>
@@ -76838,7 +77131,7 @@
       </c>
       <c r="XFD718" s="4"/>
     </row>
-    <row r="719" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="719" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A719" s="2">
         <f>HEX2DEC(D719)</f>
         <v>806568450</v>
@@ -76956,7 +77249,7 @@
       </c>
       <c r="XFD719" s="4"/>
     </row>
-    <row r="720" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="720" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A720" s="2">
         <f>HEX2DEC(D720)</f>
         <v>806569474</v>
@@ -77070,9 +77363,12 @@
       <c r="BJ720" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK720" s="6" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD720" s="4"/>
     </row>
-    <row r="721" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="721" spans="1:63 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A721" s="2">
         <f>HEX2DEC(D721)</f>
         <v>806569475</v>
@@ -77185,9 +77481,12 @@
       <c r="BJ721" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK721" s="3" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD721" s="4"/>
     </row>
-    <row r="722" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="722" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A722" s="2">
         <f>HEX2DEC(D722)</f>
         <v>806576900</v>
@@ -77300,8 +77599,11 @@
       <c r="BC722" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="723" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK722" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="723" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A723" s="2">
         <f>HEX2DEC(D723)</f>
         <v>806585090</v>
@@ -77407,7 +77709,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="724" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="724" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A724" s="2">
         <f>HEX2DEC(D724)</f>
         <v>806617345</v>
@@ -77512,7 +77814,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="725" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="725" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A725" s="2">
         <f>HEX2DEC(D725)</f>
         <v>806617346</v>
@@ -77617,7 +77919,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="726" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="726" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A726" s="2">
         <f>HEX2DEC(D726)</f>
         <v>806617602</v>
@@ -77719,7 +78021,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="727" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="727" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A727" s="2">
         <f>HEX2DEC(D727)</f>
         <v>806617857</v>
@@ -77824,7 +78126,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="728" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="728" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A728" s="2">
         <f>HEX2DEC(D728)</f>
         <v>806617858</v>
@@ -77929,7 +78231,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="729" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="729" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A729" s="2">
         <f>HEX2DEC(D729)</f>
         <v>806617859</v>
@@ -78034,7 +78336,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="730" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="730" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A730" s="2">
         <f>HEX2DEC(D730)</f>
         <v>806617860</v>
@@ -78139,7 +78441,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="731" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="731" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A731" s="2">
         <f>HEX2DEC(D731)</f>
         <v>806618116</v>
@@ -78247,7 +78549,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="732" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="732" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A732" s="2">
         <f>HEX2DEC(D732)</f>
         <v>806634753</v>
@@ -78354,8 +78656,11 @@
       <c r="BE732" s="3" t="s">
         <v>2830</v>
       </c>
-    </row>
-    <row r="733" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK732" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="733" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A733" s="2">
         <f>HEX2DEC(D733)</f>
         <v>806634754</v>
@@ -78462,8 +78767,11 @@
       <c r="BE733" s="3" t="s">
         <v>2830</v>
       </c>
-    </row>
-    <row r="734" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK733" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="734" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A734" s="2">
         <f>HEX2DEC(D734)</f>
         <v>806634755</v>
@@ -78567,8 +78875,11 @@
       <c r="AI734" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="735" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK734" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="735" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A735" s="2">
         <f>HEX2DEC(D735)</f>
         <v>806634756</v>
@@ -78672,8 +78983,11 @@
       <c r="AI735" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="736" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK735" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="736" spans="1:63 16384:16384" x14ac:dyDescent="0.4">
       <c r="A736" s="2">
         <f>HEX2DEC(D736)</f>
         <v>806635009</v>
@@ -78778,7 +79092,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="737" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="737" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A737" s="2">
         <f>HEX2DEC(D737)</f>
         <v>806635010</v>
@@ -78883,7 +79197,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="738" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="738" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A738" s="2">
         <f>HEX2DEC(D738)</f>
         <v>806650883</v>
@@ -78991,7 +79305,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="739" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="739" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A739" s="2">
         <f>HEX2DEC(D739)</f>
         <v>806683393</v>
@@ -79106,7 +79420,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="740" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="740" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A740" s="2">
         <f>HEX2DEC(D740)</f>
         <v>806683394</v>
@@ -79221,7 +79535,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="741" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="741" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A741" s="2">
         <f>HEX2DEC(D741)</f>
         <v>806686977</v>
@@ -79320,7 +79634,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="742" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="742" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A742" s="2">
         <f>HEX2DEC(D742)</f>
         <v>806686978</v>
@@ -79419,7 +79733,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="743" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="743" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A743" s="2">
         <f>HEX2DEC(D743)</f>
         <v>806686979</v>
@@ -79518,7 +79832,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="744" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="744" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A744" s="2">
         <f>HEX2DEC(D744)</f>
         <v>806686980</v>
@@ -79617,7 +79931,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="745" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="745" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A745" s="2">
         <f>HEX2DEC(D745)</f>
         <v>806699265</v>
@@ -79728,7 +80042,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="746" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="746" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A746" s="2">
         <f>HEX2DEC(D746)</f>
         <v>806699266</v>
@@ -79839,7 +80153,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="747" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="747" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A747" s="2">
         <f>HEX2DEC(D747)</f>
         <v>806699521</v>
@@ -79953,7 +80267,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="748" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="748" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A748" s="2">
         <f>HEX2DEC(D748)</f>
         <v>806699522</v>
@@ -80070,7 +80384,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="749" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="749" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A749" s="2">
         <f>HEX2DEC(D749)</f>
         <v>806716418</v>
@@ -80181,8 +80495,12 @@
       <c r="AX749" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="750" spans="1:55" x14ac:dyDescent="0.4">
+      <c r="BK749" s="3" t="s">
+        <v>2850</v>
+      </c>
+      <c r="BL749" s="3"/>
+    </row>
+    <row r="750" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A750" s="2">
         <f>HEX2DEC(D750)</f>
         <v>806724609</v>
@@ -80299,8 +80617,11 @@
       <c r="AX750" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="751" spans="1:55" x14ac:dyDescent="0.4">
+      <c r="BK750" s="3" t="s">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="751" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A751" s="2">
         <f>HEX2DEC(D751)</f>
         <v>806748417</v>
@@ -80345,7 +80666,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="752" spans="1:55" x14ac:dyDescent="0.4">
+    <row r="752" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A752" s="2">
         <f>HEX2DEC(D752)</f>
         <v>806748433</v>
@@ -80390,7 +80711,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="753" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="753" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A753" s="2">
         <f>HEX2DEC(D753)</f>
         <v>806748673</v>
@@ -80435,7 +80756,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="754" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="754" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A754" s="2">
         <f>HEX2DEC(D754)</f>
         <v>806748689</v>
@@ -80480,7 +80801,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="755" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="755" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A755" s="2">
         <f>HEX2DEC(D755)</f>
         <v>806748929</v>
@@ -80525,7 +80846,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="756" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="756" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A756" s="2">
         <f>HEX2DEC(D756)</f>
         <v>806748930</v>
@@ -80570,7 +80891,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="757" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="757" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A757" s="2">
         <f>HEX2DEC(D757)</f>
         <v>806752769</v>
@@ -80669,7 +80990,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="758" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="758" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A758" s="2">
         <f>HEX2DEC(D758)</f>
         <v>806753025</v>
@@ -80767,8 +81088,11 @@
       <c r="AI758" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="759" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BK758" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="759" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A759" s="2">
         <f>HEX2DEC(D759)</f>
         <v>806753282</v>
@@ -80870,7 +81194,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="760" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="760" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A760" s="2">
         <f>HEX2DEC(D760)</f>
         <v>806753538</v>
@@ -80972,7 +81296,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="761" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="761" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A761" s="2">
         <f>HEX2DEC(D761)</f>
         <v>806753793</v>
@@ -81074,7 +81398,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="762" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="762" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A762" s="2">
         <f>HEX2DEC(D762)</f>
         <v>806753794</v>
@@ -81176,7 +81500,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="763" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="763" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A763" s="2">
         <f>HEX2DEC(D763)</f>
         <v>806754307</v>
@@ -81274,8 +81598,11 @@
       <c r="AI763" s="1" t="s">
         <v>1353</v>
       </c>
-    </row>
-    <row r="764" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BK763" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="764" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A764" s="2">
         <f>HEX2DEC(D764)</f>
         <v>806754308</v>
@@ -81373,8 +81700,11 @@
       <c r="AI764" s="1" t="s">
         <v>1353</v>
       </c>
-    </row>
-    <row r="765" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BK764" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="765" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A765" s="2">
         <f>HEX2DEC(D765)</f>
         <v>806760705</v>
@@ -81484,8 +81814,11 @@
       <c r="BG765" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="766" spans="1:59" x14ac:dyDescent="0.4">
+      <c r="BK765" s="3" t="s">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="766" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A766" s="2">
         <f>HEX2DEC(D766)</f>
         <v>806762241</v>
@@ -81596,7 +81929,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="767" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="767" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A767" s="2">
         <f>HEX2DEC(D767)</f>
         <v>806762242</v>
@@ -81713,7 +82046,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="768" spans="1:59" x14ac:dyDescent="0.4">
+    <row r="768" spans="1:63" x14ac:dyDescent="0.4">
       <c r="A768" s="2">
         <f>HEX2DEC(D768)</f>
         <v>806762244</v>
@@ -81824,7 +82157,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="769" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="769" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A769" s="2">
         <f>HEX2DEC(D769)</f>
         <v>806888449</v>
@@ -81884,7 +82217,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="770" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="770" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A770" s="2">
         <f>HEX2DEC(D770)</f>
         <v>806945281</v>
@@ -81977,8 +82310,11 @@
       <c r="BJ770" s="3" t="s">
         <v>2841</v>
       </c>
-    </row>
-    <row r="771" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BK770" s="3" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+    <row r="771" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A771" s="2">
         <f>HEX2DEC(D771)</f>
         <v>807552769</v>
@@ -82077,7 +82413,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="772" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="772" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A772" s="2">
         <f>HEX2DEC(D772)</f>
         <v>807552771</v>
@@ -82176,7 +82512,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="773" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="773" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A773" s="2">
         <f>HEX2DEC(D773)</f>
         <v>807741441</v>
@@ -82275,7 +82611,7 @@
         <v>2637</v>
       </c>
     </row>
-    <row r="774" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="774" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A774" s="2">
         <f>HEX2DEC(D774)</f>
         <v>808732417</v>
@@ -82380,7 +82716,7 @@
         <v>2830</v>
       </c>
     </row>
-    <row r="775" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="775" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A775" s="2">
         <f>HEX2DEC(D775)</f>
         <v>808801537</v>
@@ -82483,7 +82819,7 @@
       </c>
       <c r="BA775" s="3"/>
     </row>
-    <row r="776" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="776" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A776" s="2">
         <f>HEX2DEC(D776)</f>
         <v>809572426</v>
@@ -82591,7 +82927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="777" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="777" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A777" s="2">
         <f>HEX2DEC(D777)</f>
         <v>809650176</v>
@@ -82705,7 +83041,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="778" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="778" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A778" s="2">
         <f>HEX2DEC(D778)</f>
         <v>809907475</v>
@@ -82816,7 +83152,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="779" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="779" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A779" s="2">
         <f>HEX2DEC(D779)</f>
         <v>809928706</v>
@@ -82861,7 +83197,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="780" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="780" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A780" s="2">
         <f>HEX2DEC(D780)</f>
         <v>811936001</v>
@@ -82963,7 +83299,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="781" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="781" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A781" s="2">
         <f>HEX2DEC(D781)</f>
         <v>812807202</v>
@@ -83061,8 +83397,11 @@
       <c r="AI781" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="782" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BL781" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="782" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A782" s="2">
         <f>HEX2DEC(D782)</f>
         <v>812979201</v>
@@ -83158,7 +83497,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="783" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="783" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A783" s="2">
         <f>HEX2DEC(D783)</f>
         <v>816007169</v>
@@ -83266,7 +83605,7 @@
         <v>2841</v>
       </c>
     </row>
-    <row r="784" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="784" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A784" s="2">
         <f>HEX2DEC(D784)</f>
         <v>818087685</v>
@@ -83362,7 +83701,7 @@
         <v>1216</v>
       </c>
     </row>
-    <row r="785" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="785" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A785" s="2">
         <f>HEX2DEC(D785)</f>
         <v>843466754</v>
@@ -83407,7 +83746,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="786" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="786" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A786" s="2">
         <f>HEX2DEC(D786)</f>
         <v>974537473</v>
@@ -83455,7 +83794,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="787" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="787" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A787" s="2">
         <f>HEX2DEC(D787)</f>
         <v>974537474</v>
@@ -83503,7 +83842,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="788" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="788" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A788" s="2">
         <f>HEX2DEC(D788)</f>
         <v>991049482</v>
@@ -83613,8 +83952,11 @@
       <c r="AJ788" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="789" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BL788" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="789" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A789" s="2">
         <f>HEX2DEC(D789)</f>
         <v>991127043</v>
@@ -83727,9 +84069,12 @@
       <c r="BJ789" s="6" t="s">
         <v>2841</v>
       </c>
+      <c r="BK789" s="6" t="s">
+        <v>2845</v>
+      </c>
       <c r="XFD789" s="4"/>
     </row>
-    <row r="790" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="790" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A790" s="2">
         <f>HEX2DEC(D790)</f>
         <v>991252739</v>
@@ -83839,8 +84184,14 @@
       <c r="AX790" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="791" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK790" s="3" t="s">
+        <v>2849</v>
+      </c>
+      <c r="BL790" s="3" t="s">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="791" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A791" s="2">
         <f>HEX2DEC(D791)</f>
         <v>991310850</v>
@@ -83942,7 +84293,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="792" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="792" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A792" s="2">
         <f>HEX2DEC(D792)</f>
         <v>1008029953</v>
@@ -84052,8 +84403,11 @@
       <c r="AX792" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="793" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BL792" s="3" t="s">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="793" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A793" s="2">
         <f>HEX2DEC(D793)</f>
         <v>1008029954</v>
@@ -84163,8 +84517,11 @@
       <c r="AX793" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="794" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BL793" s="3" t="s">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="794" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A794" s="2">
         <f>HEX2DEC(D794)</f>
         <v>1008029955</v>
@@ -84277,8 +84634,14 @@
       <c r="BC794" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="795" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK794" s="3" t="s">
+        <v>2849</v>
+      </c>
+      <c r="BL794" s="3" t="s">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="795" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A795" s="2">
         <f>HEX2DEC(D795)</f>
         <v>1008029956</v>
@@ -84391,8 +84754,11 @@
       <c r="BC795" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="796" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BL795" s="3" t="s">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="796" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A796" s="2">
         <f>HEX2DEC(D796)</f>
         <v>1024603157</v>
@@ -84500,7 +84866,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="797" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="797" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A797" s="2">
         <f>HEX2DEC(D797)</f>
         <v>1024603650</v>
@@ -84611,7 +84977,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="798" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="798" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A798" s="2">
         <f>HEX2DEC(D798)</f>
         <v>1024603905</v>
@@ -84719,7 +85085,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="799" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="799" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A799" s="2">
         <f>HEX2DEC(D799)</f>
         <v>1024620819</v>
@@ -84826,8 +85192,11 @@
       <c r="AI799" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="800" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BL799" s="3" t="s">
+        <v>2854</v>
+      </c>
+    </row>
+    <row r="800" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A800" s="2">
         <f>HEX2DEC(D800)</f>
         <v>1024656641</v>
@@ -84939,7 +85308,7 @@
       </c>
       <c r="XFD800" s="4"/>
     </row>
-    <row r="801" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="801" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A801" s="2">
         <f>HEX2DEC(D801)</f>
         <v>1024664065</v>
@@ -85058,7 +85427,7 @@
       </c>
       <c r="XFD801" s="4"/>
     </row>
-    <row r="802" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="802" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A802" s="2">
         <f>HEX2DEC(D802)</f>
         <v>1041662209</v>
@@ -85103,7 +85472,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="803" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="803" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A803" s="2">
         <f>HEX2DEC(D803)</f>
         <v>1041662225</v>
@@ -85148,7 +85517,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="804" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="804" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A804" s="2">
         <f>HEX2DEC(D804)</f>
         <v>1041666817</v>
@@ -85249,8 +85618,11 @@
       <c r="AI804" s="1" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="805" spans="1:62 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="BK804" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="805" spans="1:64 16384:16384" s="5" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A805" s="2">
         <f>HEX2DEC(D805)</f>
         <v>1058219265</v>
@@ -85368,7 +85740,7 @@
       </c>
       <c r="XFD805" s="4"/>
     </row>
-    <row r="806" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="806" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A806" s="2">
         <f>HEX2DEC(D806)</f>
         <v>1058301185</v>
@@ -85481,8 +85853,11 @@
       <c r="BE806" s="3" t="s">
         <v>2830</v>
       </c>
-    </row>
-    <row r="807" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK806" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="807" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A807" s="2">
         <f>HEX2DEC(D807)</f>
         <v>1058391041</v>
@@ -85600,8 +85975,11 @@
       <c r="BC807" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="808" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK807" s="3" t="s">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="808" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A808" s="2">
         <f>HEX2DEC(D808)</f>
         <v>1058414865</v>
@@ -85649,7 +86027,7 @@
         <v>2807</v>
       </c>
     </row>
-    <row r="809" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="809" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A809" s="2">
         <f>HEX2DEC(D809)</f>
         <v>1058418945</v>
@@ -85774,8 +86152,11 @@
       <c r="BG809" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="810" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK809" s="3" t="s">
+        <v>2847</v>
+      </c>
+    </row>
+    <row r="810" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A810" s="2">
         <f>HEX2DEC(D810)</f>
         <v>1058547202</v>
@@ -85834,8 +86215,11 @@
       <c r="BE810" s="3" t="s">
         <v>2830</v>
       </c>
-    </row>
-    <row r="811" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BK810" s="3" t="s">
+        <v>2845</v>
+      </c>
+    </row>
+    <row r="811" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A811" s="2">
         <f>HEX2DEC(D811)</f>
         <v>1074947586</v>
@@ -85945,8 +86329,11 @@
       <c r="BF811" s="3" t="s">
         <v>2807</v>
       </c>
-    </row>
-    <row r="812" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+      <c r="BL811" s="3" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="812" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A812" s="2">
         <f>HEX2DEC(D812)</f>
         <v>1076176897</v>
@@ -86042,7 +86429,7 @@
         <v>2733</v>
       </c>
     </row>
-    <row r="813" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="813" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A813" s="1">
         <v>2046886144</v>
       </c>
@@ -86079,7 +86466,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="814" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="814" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A814" s="1">
         <v>2046890240</v>
       </c>
@@ -86116,7 +86503,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="815" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="815" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A815" s="1">
         <v>2046984448</v>
       </c>
@@ -86153,7 +86540,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="816" spans="1:62 16384:16384" x14ac:dyDescent="0.4">
+    <row r="816" spans="1:64 16384:16384" x14ac:dyDescent="0.4">
       <c r="A816" s="1">
         <v>2046984704</v>
       </c>
@@ -90861,7 +91248,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="945" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="945" spans="1:64" x14ac:dyDescent="0.4">
       <c r="O945" s="2"/>
       <c r="P945" s="2"/>
       <c r="Q945" s="2"/>
@@ -90883,24 +91270,25 @@
       <c r="AG945" s="2"/>
       <c r="AI945" s="2"/>
       <c r="BJ945" s="3"/>
-    </row>
-    <row r="947" spans="1:62" x14ac:dyDescent="0.4">
+      <c r="BL945" s="3"/>
+    </row>
+    <row r="947" spans="1:64" x14ac:dyDescent="0.4">
       <c r="N947" s="3"/>
       <c r="P947" s="2"/>
     </row>
-    <row r="948" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="948" spans="1:64" x14ac:dyDescent="0.4">
       <c r="A948" s="2"/>
       <c r="N948" s="3"/>
       <c r="P948" s="2"/>
       <c r="Q948" s="2"/>
     </row>
-    <row r="949" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="949" spans="1:64" x14ac:dyDescent="0.4">
       <c r="N949" s="3"/>
       <c r="P949" s="2"/>
       <c r="Q949" s="2"/>
       <c r="R949" s="2"/>
     </row>
-    <row r="950" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="950" spans="1:64" x14ac:dyDescent="0.4">
       <c r="E950" s="2"/>
       <c r="F950" s="2"/>
       <c r="G950" s="2"/>
@@ -90932,7 +91320,7 @@
       <c r="AG950" s="2"/>
       <c r="AI950" s="2"/>
     </row>
-    <row r="951" spans="1:62" x14ac:dyDescent="0.4">
+    <row r="951" spans="1:64" x14ac:dyDescent="0.4">
       <c r="E951" s="2"/>
       <c r="F951" s="2"/>
       <c r="G951" s="2"/>
@@ -90965,8 +91353,8 @@
       <c r="AI951" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BJ944" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:BJ944">
+  <autoFilter ref="A2:BL944" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:BL944">
       <sortCondition ref="A2:A944"/>
     </sortState>
   </autoFilter>

</xml_diff>